<commit_message>
Open the QMS and PLM workbook on the Introduction tab
Re-saved on Introduction, so downloads land on the start-here guide
instead of the Vendors tab. Cell contents unchanged.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/files/medtech-qms-plm-vendor-evaluation-niavicta.xlsx
+++ b/files/medtech-qms-plm-vendor-evaluation-niavicta.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DE30EA8-DDD2-4C05-8091-497F4729E0A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-6340" windowWidth="38620" windowHeight="21100" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38510" yWindow="-6340" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Introduction" sheetId="1" r:id="rId1"/>
@@ -1461,25 +1461,25 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1888,14 +1888,14 @@
     <row r="1" spans="1:21" ht="52.05" customHeight="1">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
-      <c r="C1" s="28" t="s">
+      <c r="C1" s="26" t="s">
         <v>275</v>
       </c>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -2007,16 +2007,16 @@
       <c r="U5" s="1"/>
     </row>
     <row r="6" spans="1:21" ht="25.05" customHeight="1">
-      <c r="A6" s="26" t="s">
+      <c r="A6" s="27" t="s">
         <v>276</v>
       </c>
-      <c r="B6" s="27"/>
-      <c r="C6" s="27"/>
-      <c r="D6" s="27"/>
-      <c r="E6" s="27"/>
-      <c r="F6" s="27"/>
-      <c r="G6" s="27"/>
-      <c r="H6" s="27"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="28"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="28"/>
+      <c r="F6" s="28"/>
+      <c r="G6" s="28"/>
+      <c r="H6" s="28"/>
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
@@ -2180,16 +2180,16 @@
       <c r="U12" s="1"/>
     </row>
     <row r="13" spans="1:21" ht="25.05" customHeight="1">
-      <c r="A13" s="27" t="s">
+      <c r="A13" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="B13" s="27"/>
-      <c r="C13" s="27"/>
-      <c r="D13" s="27"/>
-      <c r="E13" s="27"/>
-      <c r="F13" s="27"/>
-      <c r="G13" s="27"/>
-      <c r="H13" s="27"/>
+      <c r="B13" s="28"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="28"/>
+      <c r="F13" s="28"/>
+      <c r="G13" s="28"/>
+      <c r="H13" s="28"/>
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
@@ -2205,16 +2205,16 @@
       <c r="U13" s="1"/>
     </row>
     <row r="14" spans="1:21" ht="34.049999999999997" customHeight="1">
-      <c r="A14" s="31" t="s">
+      <c r="A14" s="29" t="s">
         <v>277</v>
       </c>
-      <c r="B14" s="32"/>
-      <c r="C14" s="32"/>
-      <c r="D14" s="32"/>
-      <c r="E14" s="32"/>
-      <c r="F14" s="32"/>
-      <c r="G14" s="32"/>
-      <c r="H14" s="32"/>
+      <c r="B14" s="30"/>
+      <c r="C14" s="30"/>
+      <c r="D14" s="30"/>
+      <c r="E14" s="30"/>
+      <c r="F14" s="30"/>
+      <c r="G14" s="30"/>
+      <c r="H14" s="30"/>
       <c r="I14" s="1"/>
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
@@ -2253,16 +2253,16 @@
       <c r="U15" s="1"/>
     </row>
     <row r="16" spans="1:21" ht="25.05" customHeight="1">
-      <c r="A16" s="27" t="s">
+      <c r="A16" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="B16" s="27"/>
-      <c r="C16" s="27"/>
-      <c r="D16" s="27"/>
-      <c r="E16" s="27"/>
-      <c r="F16" s="27"/>
-      <c r="G16" s="27"/>
-      <c r="H16" s="27"/>
+      <c r="B16" s="28"/>
+      <c r="C16" s="28"/>
+      <c r="D16" s="28"/>
+      <c r="E16" s="28"/>
+      <c r="F16" s="28"/>
+      <c r="G16" s="28"/>
+      <c r="H16" s="28"/>
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
       <c r="K16" s="1"/>
@@ -2281,15 +2281,15 @@
       <c r="A17" s="1">
         <v>0</v>
       </c>
-      <c r="B17" s="30" t="s">
+      <c r="B17" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="C17" s="30"/>
-      <c r="D17" s="30"/>
-      <c r="E17" s="30"/>
-      <c r="F17" s="30"/>
-      <c r="G17" s="30"/>
-      <c r="H17" s="30"/>
+      <c r="C17" s="31"/>
+      <c r="D17" s="31"/>
+      <c r="E17" s="31"/>
+      <c r="F17" s="31"/>
+      <c r="G17" s="31"/>
+      <c r="H17" s="31"/>
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
       <c r="K17" s="1"/>
@@ -2308,15 +2308,15 @@
       <c r="A18" s="1">
         <v>1</v>
       </c>
-      <c r="B18" s="30" t="s">
+      <c r="B18" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="30"/>
-      <c r="D18" s="30"/>
-      <c r="E18" s="30"/>
-      <c r="F18" s="30"/>
-      <c r="G18" s="30"/>
-      <c r="H18" s="30"/>
+      <c r="C18" s="31"/>
+      <c r="D18" s="31"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="31"/>
+      <c r="G18" s="31"/>
+      <c r="H18" s="31"/>
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
@@ -2335,15 +2335,15 @@
       <c r="A19" s="1">
         <v>2</v>
       </c>
-      <c r="B19" s="30" t="s">
+      <c r="B19" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="C19" s="30"/>
-      <c r="D19" s="30"/>
-      <c r="E19" s="30"/>
-      <c r="F19" s="30"/>
-      <c r="G19" s="30"/>
-      <c r="H19" s="30"/>
+      <c r="C19" s="31"/>
+      <c r="D19" s="31"/>
+      <c r="E19" s="31"/>
+      <c r="F19" s="31"/>
+      <c r="G19" s="31"/>
+      <c r="H19" s="31"/>
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
       <c r="K19" s="1"/>
@@ -2362,15 +2362,15 @@
       <c r="A20" s="1">
         <v>3</v>
       </c>
-      <c r="B20" s="30" t="s">
+      <c r="B20" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="C20" s="30"/>
-      <c r="D20" s="30"/>
-      <c r="E20" s="30"/>
-      <c r="F20" s="30"/>
-      <c r="G20" s="30"/>
-      <c r="H20" s="30"/>
+      <c r="C20" s="31"/>
+      <c r="D20" s="31"/>
+      <c r="E20" s="31"/>
+      <c r="F20" s="31"/>
+      <c r="G20" s="31"/>
+      <c r="H20" s="31"/>
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
@@ -2389,15 +2389,15 @@
       <c r="A21" s="1">
         <v>4</v>
       </c>
-      <c r="B21" s="30" t="s">
+      <c r="B21" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="C21" s="30"/>
-      <c r="D21" s="30"/>
-      <c r="E21" s="30"/>
-      <c r="F21" s="30"/>
-      <c r="G21" s="30"/>
-      <c r="H21" s="30"/>
+      <c r="C21" s="31"/>
+      <c r="D21" s="31"/>
+      <c r="E21" s="31"/>
+      <c r="F21" s="31"/>
+      <c r="G21" s="31"/>
+      <c r="H21" s="31"/>
       <c r="I21" s="1"/>
       <c r="J21" s="1"/>
       <c r="K21" s="1"/>
@@ -2416,15 +2416,15 @@
       <c r="A22" s="1">
         <v>5</v>
       </c>
-      <c r="B22" s="30" t="s">
+      <c r="B22" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="C22" s="30"/>
-      <c r="D22" s="30"/>
-      <c r="E22" s="30"/>
-      <c r="F22" s="30"/>
-      <c r="G22" s="30"/>
-      <c r="H22" s="30"/>
+      <c r="C22" s="31"/>
+      <c r="D22" s="31"/>
+      <c r="E22" s="31"/>
+      <c r="F22" s="31"/>
+      <c r="G22" s="31"/>
+      <c r="H22" s="31"/>
       <c r="I22" s="1"/>
       <c r="J22" s="1"/>
       <c r="K22" s="1"/>
@@ -2536,16 +2536,16 @@
       <c r="U26" s="1"/>
     </row>
     <row r="27" spans="1:21" ht="25.05" customHeight="1">
-      <c r="A27" s="27" t="s">
+      <c r="A27" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="B27" s="27"/>
-      <c r="C27" s="27"/>
-      <c r="D27" s="27"/>
-      <c r="E27" s="27"/>
-      <c r="F27" s="27"/>
-      <c r="G27" s="27"/>
-      <c r="H27" s="27"/>
+      <c r="B27" s="28"/>
+      <c r="C27" s="28"/>
+      <c r="D27" s="28"/>
+      <c r="E27" s="28"/>
+      <c r="F27" s="28"/>
+      <c r="G27" s="28"/>
+      <c r="H27" s="28"/>
       <c r="I27" s="1"/>
       <c r="J27" s="1"/>
       <c r="K27" s="1"/>
@@ -2659,16 +2659,16 @@
       <c r="U31" s="1"/>
     </row>
     <row r="32" spans="1:21" ht="25.05" customHeight="1">
-      <c r="A32" s="27" t="s">
+      <c r="A32" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="B32" s="27"/>
-      <c r="C32" s="27"/>
-      <c r="D32" s="27"/>
-      <c r="E32" s="27"/>
-      <c r="F32" s="27"/>
-      <c r="G32" s="27"/>
-      <c r="H32" s="27"/>
+      <c r="B32" s="28"/>
+      <c r="C32" s="28"/>
+      <c r="D32" s="28"/>
+      <c r="E32" s="28"/>
+      <c r="F32" s="28"/>
+      <c r="G32" s="28"/>
+      <c r="H32" s="28"/>
       <c r="I32" s="1"/>
       <c r="J32" s="1"/>
       <c r="K32" s="1"/>
@@ -2757,7 +2757,7 @@
       <c r="U35" s="1"/>
     </row>
     <row r="36" spans="1:21" ht="43.95" customHeight="1">
-      <c r="A36" s="29" t="s">
+      <c r="A36" s="32" t="s">
         <v>278</v>
       </c>
       <c r="B36" s="25"/>
@@ -2782,7 +2782,7 @@
       <c r="U36" s="1"/>
     </row>
     <row r="37" spans="1:21" ht="43.95" customHeight="1">
-      <c r="A37" s="29" t="s">
+      <c r="A37" s="32" t="s">
         <v>279</v>
       </c>
       <c r="B37" s="25"/>
@@ -2807,7 +2807,7 @@
       <c r="U37" s="1"/>
     </row>
     <row r="38" spans="1:21" ht="43.95" customHeight="1">
-      <c r="A38" s="29" t="s">
+      <c r="A38" s="32" t="s">
         <v>280</v>
       </c>
       <c r="B38" s="25"/>
@@ -2832,7 +2832,7 @@
       <c r="U38" s="1"/>
     </row>
     <row r="39" spans="1:21" ht="43.95" customHeight="1">
-      <c r="A39" s="29" t="s">
+      <c r="A39" s="32" t="s">
         <v>281</v>
       </c>
       <c r="B39" s="25"/>
@@ -4238,36 +4238,36 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="A34:H34"/>
+    <mergeCell ref="A36:H36"/>
+    <mergeCell ref="A37:H37"/>
+    <mergeCell ref="A38:H38"/>
+    <mergeCell ref="A39:H39"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A30:H30"/>
+    <mergeCell ref="A32:H32"/>
+    <mergeCell ref="A33:H33"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="B22:H22"/>
+    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="B17:H17"/>
+    <mergeCell ref="B18:H18"/>
+    <mergeCell ref="B19:H19"/>
+    <mergeCell ref="B20:H20"/>
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A14:H14"/>
     <mergeCell ref="C1:H1"/>
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="A6:H6"/>
     <mergeCell ref="A7:H7"/>
     <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A9:H9"/>
-    <mergeCell ref="A10:H10"/>
-    <mergeCell ref="A11:H11"/>
-    <mergeCell ref="A13:H13"/>
-    <mergeCell ref="A14:H14"/>
-    <mergeCell ref="A16:H16"/>
-    <mergeCell ref="B17:H17"/>
-    <mergeCell ref="B18:H18"/>
-    <mergeCell ref="B19:H19"/>
-    <mergeCell ref="B20:H20"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="B22:H22"/>
-    <mergeCell ref="A24:H24"/>
-    <mergeCell ref="A25:H25"/>
-    <mergeCell ref="A27:H27"/>
-    <mergeCell ref="A28:H28"/>
-    <mergeCell ref="A29:H29"/>
-    <mergeCell ref="A30:H30"/>
-    <mergeCell ref="A32:H32"/>
-    <mergeCell ref="A33:H33"/>
-    <mergeCell ref="A34:H34"/>
-    <mergeCell ref="A36:H36"/>
-    <mergeCell ref="A37:H37"/>
-    <mergeCell ref="A38:H38"/>
-    <mergeCell ref="A39:H39"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -4291,14 +4291,14 @@
     <row r="1" spans="1:21" ht="52.05" customHeight="1">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
-      <c r="C1" s="28" t="s">
+      <c r="C1" s="26" t="s">
         <v>275</v>
       </c>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -5096,19 +5096,19 @@
       <c r="U18" s="1"/>
     </row>
     <row r="19" spans="1:21" ht="25.05" customHeight="1">
-      <c r="A19" s="26" t="s">
+      <c r="A19" s="27" t="s">
         <v>282</v>
       </c>
-      <c r="B19" s="27"/>
-      <c r="C19" s="27"/>
-      <c r="D19" s="27"/>
-      <c r="E19" s="27"/>
-      <c r="F19" s="27"/>
-      <c r="G19" s="27"/>
-      <c r="H19" s="27"/>
-      <c r="I19" s="27"/>
-      <c r="J19" s="27"/>
-      <c r="K19" s="27"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="28"/>
+      <c r="F19" s="28"/>
+      <c r="G19" s="28"/>
+      <c r="H19" s="28"/>
+      <c r="I19" s="28"/>
+      <c r="J19" s="28"/>
+      <c r="K19" s="28"/>
       <c r="L19" s="1"/>
       <c r="M19" s="1"/>
       <c r="N19" s="1"/>
@@ -5607,20 +5607,20 @@
       <c r="U29" s="1"/>
     </row>
     <row r="30" spans="1:21" ht="25.05" customHeight="1">
-      <c r="A30" s="26" t="s">
+      <c r="A30" s="27" t="s">
         <v>283</v>
       </c>
-      <c r="B30" s="27"/>
-      <c r="C30" s="27"/>
-      <c r="D30" s="27"/>
-      <c r="E30" s="27"/>
-      <c r="F30" s="27"/>
-      <c r="G30" s="27"/>
-      <c r="H30" s="27"/>
-      <c r="I30" s="27"/>
-      <c r="J30" s="27"/>
-      <c r="K30" s="27"/>
-      <c r="L30" s="27"/>
+      <c r="B30" s="28"/>
+      <c r="C30" s="28"/>
+      <c r="D30" s="28"/>
+      <c r="E30" s="28"/>
+      <c r="F30" s="28"/>
+      <c r="G30" s="28"/>
+      <c r="H30" s="28"/>
+      <c r="I30" s="28"/>
+      <c r="J30" s="28"/>
+      <c r="K30" s="28"/>
+      <c r="L30" s="28"/>
       <c r="M30" s="1"/>
       <c r="N30" s="1"/>
       <c r="O30" s="1"/>

</xml_diff>